<commit_message>
feat(client/server): implementar ventana de configuracion (Settings) y edicion visual de conductores/vehiculos (RF-11)
</commit_message>
<xml_diff>
--- a/docs/Diccionario_Datos_V2_Sincronizado.xlsx
+++ b/docs/Diccionario_Datos_V2_Sincronizado.xlsx
@@ -10,10 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Driver" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vehicle" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RateTariff" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trip" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RefreshToken" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trip" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RefreshToken" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -484,7 +483,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Identificador Único Universal (UUID).</t>
+          <t>Identificador Único Universal (UUID) autogenerado.</t>
         </is>
       </c>
     </row>
@@ -507,7 +506,7 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Datos personales registrados en el sistema.</t>
+          <t>Parte de la información del nombre personal (primerNombre).</t>
         </is>
       </c>
     </row>
@@ -530,7 +529,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Datos personales registrados en el sistema.</t>
+          <t>Parte de la información del nombre personal (segundoNombre).</t>
         </is>
       </c>
     </row>
@@ -553,7 +552,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Datos personales registrados en el sistema.</t>
+          <t>Parte de la información del nombre personal (primerApellido).</t>
         </is>
       </c>
     </row>
@@ -576,7 +575,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Datos personales registrados en el sistema.</t>
+          <t>Parte de la información del nombre personal (segundoApellido).</t>
         </is>
       </c>
     </row>
@@ -603,7 +602,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Email único para autenticación y notificaciones.</t>
+          <t>Correo electrónico corporativo único para autenticación.</t>
         </is>
       </c>
     </row>
@@ -626,7 +625,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Hash bcrypt de seguridad para la contraseña.</t>
+          <t>Hash bcrypt de seguridad para la contraseña del usuario.</t>
         </is>
       </c>
     </row>
@@ -649,7 +648,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad User.</t>
+          <t>Rol asignado para control de acceso (ADMIN, OPERADOR).</t>
         </is>
       </c>
     </row>
@@ -672,7 +671,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Estado de activación lógica en el sistema.</t>
+          <t>Indicador lógico de activación en el sistema.</t>
         </is>
       </c>
     </row>
@@ -695,7 +694,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad User.</t>
+          <t>Marca temporal inmutable de la creación del registro.</t>
         </is>
       </c>
     </row>
@@ -718,7 +717,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad User.</t>
+          <t>Marca temporal de la última modificación automática del registro.</t>
         </is>
       </c>
     </row>
@@ -741,7 +740,7 @@
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Técnica que permite desactivar registros sin eliminarlos físicamente para garantizar la trazabilidad.</t>
+          <t>Fecha de eliminación lógica (Soft Delete) para preservar la trazabilidad.</t>
         </is>
       </c>
     </row>
@@ -909,7 +908,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Identificador Único Universal (UUID).</t>
+          <t>Identificador Único Universal (UUID) autogenerado.</t>
         </is>
       </c>
     </row>
@@ -936,7 +935,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad Driver.</t>
+          <t>Cédula de ciudadanía o identificación del conductor.</t>
         </is>
       </c>
     </row>
@@ -959,7 +958,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Datos personales registrados en el sistema.</t>
+          <t>Parte de la información del nombre personal (primerNombre).</t>
         </is>
       </c>
     </row>
@@ -982,7 +981,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Datos personales registrados en el sistema.</t>
+          <t>Parte de la información del nombre personal (segundoNombre).</t>
         </is>
       </c>
     </row>
@@ -1005,7 +1004,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Datos personales registrados en el sistema.</t>
+          <t>Parte de la información del nombre personal (primerApellido).</t>
         </is>
       </c>
     </row>
@@ -1028,7 +1027,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Datos personales registrados en el sistema.</t>
+          <t>Parte de la información del nombre personal (segundoApellido).</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1050,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad Driver.</t>
+          <t>Número telefónico de contacto del conductor.</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1073,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Estado de activación lógica en el sistema.</t>
+          <t>Indicador lógico de activación en el sistema.</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1096,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad Driver.</t>
+          <t>Marca temporal inmutable de la creación del registro.</t>
         </is>
       </c>
     </row>
@@ -1120,7 +1119,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad Driver.</t>
+          <t>Marca temporal de la última modificación automática del registro.</t>
         </is>
       </c>
     </row>
@@ -1143,7 +1142,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Técnica que permite desactivar registros sin eliminarlos físicamente para garantizar la trazabilidad.</t>
+          <t>Fecha de eliminación lógica (Soft Delete) para preservar la trazabilidad.</t>
         </is>
       </c>
     </row>
@@ -1234,7 +1233,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Identificador Único Universal (UUID).</t>
+          <t>Identificador Único Universal (UUID) autogenerado.</t>
         </is>
       </c>
     </row>
@@ -1261,7 +1260,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Identificación vehicular (Formato AAA000).</t>
+          <t>Placa patente de identificación única del vehículo.</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1283,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad Vehicle.</t>
+          <t>Marca fabricante del vehículo.</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1306,7 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad Vehicle.</t>
+          <t>Modelo o año del vehículo.</t>
         </is>
       </c>
     </row>
@@ -1330,7 +1329,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Carga máxima permitida en toneladas.</t>
+          <t>Capacidad máxima de carga permitida en toneladas métricas.</t>
         </is>
       </c>
     </row>
@@ -1353,7 +1352,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Estado operativo actual del recurso.</t>
+          <t>Estado de disponibilidad del vehículo (DISPONIBLE, EN_VIAJE, MANTENIMIENTO).</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1375,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Estado de activación lógica en el sistema.</t>
+          <t>Indicador lógico de activación en el sistema.</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1398,7 @@
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad Vehicle.</t>
+          <t>Marca temporal inmutable de la creación del registro.</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1421,7 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad Vehicle.</t>
+          <t>Marca temporal de la última modificación automática del registro.</t>
         </is>
       </c>
     </row>
@@ -1445,7 +1444,7 @@
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Técnica que permite desactivar registros sin eliminarlos físicamente para garantizar la trazabilidad.</t>
+          <t>Fecha de eliminación lógica (Soft Delete) para preservar la trazabilidad.</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1521,7 +1520,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1536,19 +1535,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Identificador Único Universal (UUID).</t>
+          <t>Identificador Único Universal (UUID) autogenerado.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>producto</t>
+          <t>ticket</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ProductType</t>
+          <t>Int</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1563,19 +1562,19 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RateTariff.</t>
+          <t>Número secuencial único del ticket de báscula física.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>valorKg</t>
+          <t>fecha</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1586,19 +1585,19 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RateTariff.</t>
+          <t>Fecha y hora en que se realizó el flete.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>activo</t>
+          <t>origen</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1609,19 +1608,19 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Estado de activación lógica en el sistema.</t>
+          <t>Ubicación de origen/cargue del flete.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>createdAt</t>
+          <t>producto</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>ProductType</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1632,19 +1631,19 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RateTariff.</t>
+          <t>Tipo de producto transportado (FRUTO, COMPOST).</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>updatedAt</t>
+          <t>tonelaje</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1655,30 +1654,483 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RateTariff.</t>
+          <t>Peso neto transportado en toneladas métricas.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>deletedAt</t>
+          <t>valorPago</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Decimal</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Técnica que permite desactivar registros sin eliminarlos físicamente para garantizar la trazabilidad.</t>
+          <t>Monto total liquidado y a pagar por el viaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>consumoAcpm</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Consumo de combustible ACPM en galones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>usoFerry</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Boolean</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Indicador de si se utilizó servicio de cruce fluvial en Ferry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>destino</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ubicación de destino del flete.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>empresa</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Nombre de la empresa destinataria o relacionada con el viaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>porcentajeConductor</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Porcentaje de comisión asignado al conductor (ej. 1.00 para 100%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>valorConductor</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Monto liquidado correspondiente al pago del conductor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>valorAcpm</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Costo monetario del combustible ACPM consumido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>valorFerry</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Decimal</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Costo monetario del cruce fluvial en Ferry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>driverId</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Clave foránea que referencia al conductor del viaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>driver</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Driver</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Relación con la entidad Conductor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>vehicleId</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Clave foránea que referencia al vehículo del viaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>vehicle</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Vehicle</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Relación con la entidad Vehículo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>registradoPorId</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Clave foránea del usuario operador que registró el viaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>registradoPor</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Relación con el Usuario creador.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>actualizadoPorId</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>String</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Clave foránea del último usuario que modificó el viaje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>actualizadoPor</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Relación con el Usuario editor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>createdAt</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Marca temporal inmutable de la creación del registro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>updatedAt</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Marca temporal de la última modificación automática del registro.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>deletedAt</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DateTime</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Fecha de eliminación lógica (Soft Delete) para preservar la trazabilidad.</t>
         </is>
       </c>
     </row>
@@ -1693,7 +2145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1746,69 +2198,69 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Identificador Único Universal (UUID).</t>
+          <t>Identificador Único Universal (UUID) autogenerado.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ticket</t>
+          <t>userId</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Int</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Unique</t>
-        </is>
-      </c>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (ticket).</t>
+          <t>Clave foránea del usuario que realizó la acción auditada.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>fecha</t>
+          <t>user</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>User</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>FK</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (fecha).</t>
+          <t>Relación con el Usuario que ejecutó la acción.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>origen</t>
+          <t>action</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>AuditAction</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1819,19 +2271,19 @@
       <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (origen).</t>
+          <t>Acción registrada (CREATE, UPDATE, DELETE, LOGIN, LOGOUT).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>producto</t>
+          <t>entity</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ProductType</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1842,88 +2294,88 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (producto).</t>
+          <t>Nombre de la entidad o tabla donde se realizó el cambio.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>tipoPago</t>
+          <t>entityId</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PaymentType</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (tipoPago).</t>
+          <t>Identificador del registro de la entidad afectada.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tonelaje</t>
+          <t>oldValues</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Json</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (tonelaje).</t>
+          <t>Estado anterior del registro en formato JSON.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>valorPago</t>
+          <t>newValues</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>Json</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (valorPago).</t>
+          <t>Estado posterior del registro en formato JSON.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>consumoAcpm</t>
+          <t>ipAddress</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Decimal</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1934,42 +2386,42 @@
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (consumoAcpm).</t>
+          <t>Dirección IP del cliente que generó el cambio.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>usoFerry</t>
+          <t>userAgent</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Boolean</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (usoFerry).</t>
+          <t>Cadena identificadora del cliente o navegador (User-Agent).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>driverId</t>
+          <t>createdAt</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>String</t>
+          <t>DateTime</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1980,253 +2432,7 @@
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Campo del Registro de Viajes y control de tickets (driverId).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>driver</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Driver</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (driver).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>vehicleId</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (vehicleId).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>vehicle</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Vehicle</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (vehicle).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>registradoPorId</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (registradoPorId).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>registradoPor</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (registradoPor).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>actualizadoPorId</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (actualizadoPorId).</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>actualizadoPor</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (actualizadoPor).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>createdAt</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (createdAt).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>updatedAt</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>Campo del Registro de Viajes y control de tickets (updatedAt).</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>deletedAt</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Técnica que permite desactivar registros sin eliminarlos físicamente para garantizar la trazabilidad.</t>
+          <t>Marca temporal inmutable de la creación del registro.</t>
         </is>
       </c>
     </row>
@@ -2241,308 +2447,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Campo</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Tipo de Dato</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Nulidad</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Clave</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Descripción Funcional</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>PK</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Identificador Único Universal (UUID).</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>userId</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (userId).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>user</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>User</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>FK</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (user).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>action</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>AuditAction</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (action).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>entity</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (entity).</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>entityId</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (entityId).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>oldValues</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Json</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (oldValues).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>newValues</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Json</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (newValues).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ipAddress</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (ipAddress).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>userAgent</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>String</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (userAgent).</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>createdAt</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>DateTime</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>Parte de la Auditoría para registrar acciones realizadas por los usuarios (createdAt).</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -2596,7 +2500,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Identificador Único Universal (UUID).</t>
+          <t>Identificador Único Universal (UUID) autogenerado.</t>
         </is>
       </c>
     </row>
@@ -2623,7 +2527,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RefreshToken.</t>
+          <t>Valor del token de refresco JWT.</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2550,7 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RefreshToken.</t>
+          <t>Clave foránea del usuario al que pertenece la sesión.</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2577,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RefreshToken.</t>
+          <t>Relación con el Usuario de la sesión.</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2600,7 @@
       <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RefreshToken.</t>
+          <t>Fecha y hora de expiración de la sesión.</t>
         </is>
       </c>
     </row>
@@ -2719,7 +2623,7 @@
       <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RefreshToken.</t>
+          <t>Indicador de si el token de refresco fue invalidado/cerrado.</t>
         </is>
       </c>
     </row>
@@ -2742,7 +2646,7 @@
       <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Atributo técnico de la entidad RefreshToken.</t>
+          <t>Marca temporal inmutable de la creación del registro.</t>
         </is>
       </c>
     </row>

</xml_diff>